<commit_message>
test(qa): split deep re-verification into new rows instead of overwriting
The previous commit (6143b7f) had overwritten TC-018/020/024's original
one-shot-test results with the deeper disposable-account re-test results,
losing the record of what the first pass actually found. Given this file
already lost real history once to a silent overwrite, that's the wrong
pattern even for a legitimate re-test by the same person.

- TC-018, TC-020, TC-024 restored to their original (first-pass) content
  and results, each with a remark pointing to its deep-test counterpart.
- Added TC-059, TC-060, TC-061 as the deep re-verification results
  (disposable throwaway account, the session-revocation bypass finding,
  the unauthenticated /api/health finding), each remarking which TC-0XX
  it re-verifies.

61 total, all unique IDs, no duplicates. 52 Passed, 1 Blocked, 8 Failed.
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -630,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" style="9" min="1" max="1"/>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>DEEPENED with a controlled single-variable test (previous check mixed in other API calls). Fresh login as the throwaway user -&gt; TTL=3600 immediately. Waited 5s, then called a NON-/me endpoint (GET /api/health) -&gt; TTL read 3595, i.e. a plain 5s countdown, NOT a reset to 3600. Confirms precisely: only /api/auth/me (and login) extend the session (rust/auth-service/src/routes/me.rs:48 is the only other .expire(&amp;session_key,...) call besides login.rs); every other authenticated call does not. So idle timeout is real but only as accurate as however often the frontend calls /me as a heartbeat.</t>
+          <t>A real sliding-window idle timeout does exist, verified live via the Valkey session TTL (not by waiting out the full window, which is impractical here). Session key provigil:session:&lt;jti&gt; is created with TTL=token_ttl (3600s) at login and is the sole gate auth-service's auth() helper checks (EXISTS). rust/auth-service/src/routes/me.rs:48 resets that TTL back to the full 3600s on every /api/auth/me call. Live check: TTL read 3477, then after 2 /api/auth/me calls 8s later it read 3600 (reset, not just counted down); a separate check 3s apart with no /me call showed a normal 3575-&gt;3572 countdown. So a session with no /me heartbeat for 3600s will fail the EXISTS check and every subsequent call gets 401, matching the expected result.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>Claude (live API test, disposable throwaway user 'qa-deep-test-01', https://localhost)</t>
+          <t>Claude (live API test, tenant_admin account 'tenant-admin', https://localhost)</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>Mechanism confirmed precisely with an isolated single-call test, not just the earlier mixed-call observation.</t>
+          <t>Verified via live TTL behavior + source, not a full 1-hour wait for the 401 itself. | See TC-059 for a deeper re-verification using a disposable test account.</t>
         </is>
       </c>
     </row>
@@ -2167,12 +2167,12 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>DEEPENED: created a disposable throwaway analyst user (qa-deep-test-01) instead of reusing testuser12, to test the full expected result end to end without touching a real account. Logged in as it, then as tenant_admin called DELETE /api/admin/sessions/qa-deep-test-01 -&gt; HTTP 200 {"sessions_terminated":1}. Re-checked the SAME old token immediately after -&gt; GET /api/auth/me still returned HTTP 200, not 401. Root cause found: force_logout_user (rust/ndr-engine/src/api/mod.rs:10500) only deletes the ndr:session:&lt;jti&gt; key. Verified directly in Valkey: after revoke, EXISTS ndr:session:&lt;jti&gt;=0 (gone) but EXISTS provigil:session:&lt;jti&gt;=1 (still there) — that second key is the ONLY one auth-service's auth() check (login/me/users/tenants routes) ever looks at, so the token keeps working there. Worse: called POST /api/auth/refresh with the 'revoked' token -&gt; HTTP 200, issued a brand-new token+jti, which login.rs's refresh path also re-writes into ndr:session: — fully restoring ndr-engine API access too. So a 'force logged out' user can undo the entire revoke with a single refresh call.</t>
+          <t>DELETE /api/admin/sessions/testuser12 (tenant_admin token, target user in own tenant) -&gt; HTTP 200 {"sessions_terminated":0,"status":"ok"} (0 because testuser12 had no active session at test time, not a failure). Endpoint exists (rust/ndr-engine api::force_logout_user) and tenant_admin is correctly allowed to revoke a same-tenant user's sessions.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>Claude (live API test, disposable throwaway user 'qa-deep-test-01', https://localhost)</t>
+          <t>Claude (live API test, tenant_admin account 'tenant-admin', https://localhost)</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>Real, reproducible security bug: session revocation only clears one of the two session-key namespaces (ndr:session: vs provigil:session:) and is fully bypassable via /api/auth/refresh. Not something I changed — flagging for a fix decision.</t>
+          <t>Partial: couldn't verify the 'old token now returns 401' half — needs testuser12's own live token/password, which wasn't available. | See TC-060 for a deeper re-verification using a disposable test account.</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>DEEPENED: tested with 3 different callers instead of one. (1) tenant_admin token -&gt; HTTP 200, full data. (2) disposable analyst token -&gt; HTTP 200, IDENTICAL full data (services status, hits_total, sigma_rules count, total event counts). (3) NO Authorization header at all -&gt; HTTP 200, the exact same response. This is not a role-scoping gap, it's fully unauthenticated: anyone who can reach https://localhost/api/health gets Kafka/ClickHouse/engine status and platform-wide counters with zero credentials. Confirmed in rust/ndr-engine/src/api/mod.rs: the handler calls extract_claims() (returns None gracefully) but has no check that requires claims to be Some, let alone a specific role.</t>
+          <t>GET /api/health with the tenant_admin token -&gt; HTTP 200 with full service status (clickhouse/kafka/engine running, event counts, sigma_rules, sessions). Expected result says tenant_admin should get 403 Forbidden on an admin health endpoint. In reality there is no /api/admin/health route at all — only /api/health exists, and rust/ndr-engine/src/api/mod.rs shows it has no role check; any authenticated caller gets the same data. The per-tenant event counts ARE correctly scoped to the caller's own tenant, but the service-status section (kafka/clickhouse/engine up-or-down) is not tenant-admin-restricted as this test expects.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>Claude (live API test, disposable throwaway user 'qa-deep-test-01', https://localhost)</t>
+          <t>Claude (live API test, tenant_admin account 'tenant-admin', https://localhost)</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>Escalating from earlier finding: this isn't just 'tenant_admin gets it when it should be 403' — the endpoint has no auth requirement whatsoever. Worth a decision on whether this is intended (a public health check) or a real gap.</t>
+          <t>Actual behavior doesn't match this test's documented expectation — worth a decision on whether /api/health should be admin-gated or this test's expectation should be revised, not something I changed unilaterally. | See TC-061 for a deeper re-verification using a disposable test account.</t>
         </is>
       </c>
     </row>
@@ -5143,6 +5143,246 @@
       <c r="O59" s="4" t="inlineStr">
         <is>
           <t>[Verification Method: Manual (live, isolated container) | Iterations: 1] No defect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="60" customHeight="1" s="9">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>TC-059</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Auth / Access Control</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Super Admin session auto-expires after inactivity</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>[Deep re-verification of TC-018] Super Admin JWT is invalidated after the configured idle timeout</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Verify that an inactive super_admin session does not remain valid indefinitely — critical to prevent privilege persistence if a session is hijacked or left unattended.</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>super_admin is logged in; session timeout is configured (e.g. 30 min)</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>1. Log in as super_admin and obtain a session token
+2. Wait for the configured idle timeout period without any activity
+3. Attempt to call a protected endpoint using the old token
+4. Observe the response</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Idle period = configured timeout value; token from step 1</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized is returned after timeout; re-authentication is required to continue</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>DEEPENED with a controlled single-variable test (previous check mixed in other API calls). Fresh login as the throwaway user -&gt; TTL=3600 immediately. Waited 5s, then called a NON-/me endpoint (GET /api/health) -&gt; TTL read 3595, i.e. a plain 5s countdown, NOT a reset to 3600. Confirms precisely: only /api/auth/me (and login) extend the session (rust/auth-service/src/routes/me.rs:48 is the only other .expire(&amp;session_key,...) call besides login.rs); every other authenticated call does not. So idle timeout is real but only as accurate as however often the frontend calls /me as a heartbeat.</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t>Claude (live API test, disposable throwaway user 'qa-deep-test-01', https://localhost)</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O60" s="4" t="inlineStr">
+        <is>
+          <t>Deep re-test of TC-018 using a disposable throwaway account (qa-deep-test-01) instead of single one-shot calls against real accounts. Mechanism confirmed precisely with an isolated single-call test, not just the earlier mixed-call observation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="60" customHeight="1" s="9">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>TC-060</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>User Management</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Super Admin force-revokes all sessions of a user</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>[Deep re-verification of TC-020] POST /api/admin/users/:id/revoke-sessions invalidates every active token</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Verify that super_admin can force-logout any user across all devices by revoking their active sessions — critical for incident response when an account is suspected to be compromised.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Target user is logged in on at least one device (active JWT exists); authenticated as super_admin</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>1. Obtain a valid session token for the target user
+2. POST /api/admin/users/:id/revoke-sessions as super_admin
+3. Confirm HTTP 200
+4. Attempt an API call using the old target-user token</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>target user_id; existing JWT of that user</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 on revoke; subsequent API calls with the old token return 401 Unauthorized; user must re-authenticate to continue</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>DEEPENED: created a disposable throwaway analyst user (qa-deep-test-01) instead of reusing testuser12, to test the full expected result end to end without touching a real account. Logged in as it, then as tenant_admin called DELETE /api/admin/sessions/qa-deep-test-01 -&gt; HTTP 200 {"sessions_terminated":1}. Re-checked the SAME old token immediately after -&gt; GET /api/auth/me still returned HTTP 200, not 401. Root cause found: force_logout_user (rust/ndr-engine/src/api/mod.rs:10500) only deletes the ndr:session:&lt;jti&gt; key. Verified directly in Valkey: after revoke, EXISTS ndr:session:&lt;jti&gt;=0 (gone) but EXISTS provigil:session:&lt;jti&gt;=1 (still there) — that second key is the ONLY one auth-service's auth() check (login/me/users/tenants routes) ever looks at, so the token keeps working there. Worse: called POST /api/auth/refresh with the 'revoked' token -&gt; HTTP 200, issued a brand-new token+jti, which login.rs's refresh path also re-writes into ndr:session: — fully restoring ndr-engine API access too. So a 'force logged out' user can undo the entire revoke with a single refresh call.</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>Claude (live API test, disposable throwaway user 'qa-deep-test-01', https://localhost)</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t>Deep re-test of TC-020 using a disposable throwaway account (qa-deep-test-01) instead of single one-shot calls against real accounts. Real, reproducible security bug: session revocation only clears one of the two session-key namespaces (ndr:session: vs provigil:session:) and is fully bypassable via /api/auth/refresh. Not something I changed — flagging for a fix decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="60" customHeight="1" s="9">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>TC-061</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>System Monitoring</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Super Admin views real-time system health dashboard</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>[Deep re-verification of TC-024] GET /api/admin/health returns live metrics for all services</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Verify that super_admin can access a system health endpoint that reports live status of all core services (ndr-engine, auth-service, database, message queue) and that tenant_admin is denied access.</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>All core services are running; authenticated as super_admin</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>1. GET /api/admin/health as super_admin
+2. Confirm HTTP 200 and response includes status for each service
+3. Check for fields: service name, status (up/down), latency, uptime
+4. Repeat request as tenant_admin and confirm 403</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>Super Admin: HTTP 200 with per-service health data. Tenant Admin: HTTP 403 Forbidden. All running services report status='up'</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>DEEPENED: tested with 3 different callers instead of one. (1) tenant_admin token -&gt; HTTP 200, full data. (2) disposable analyst token -&gt; HTTP 200, IDENTICAL full data (services status, hits_total, sigma_rules count, total event counts). (3) NO Authorization header at all -&gt; HTTP 200, the exact same response. This is not a role-scoping gap, it's fully unauthenticated: anyone who can reach https://localhost/api/health gets Kafka/ClickHouse/engine status and platform-wide counters with zero credentials. Confirmed in rust/ndr-engine/src/api/mod.rs: the handler calls extract_claims() (returns None gracefully) but has no check that requires claims to be Some, let alone a specific role.</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t>Claude (live API test, disposable throwaway user 'qa-deep-test-01', https://localhost)</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O62" s="4" t="inlineStr">
+        <is>
+          <t>Deep re-test of TC-024 using a disposable throwaway account (qa-deep-test-01) instead of single one-shot calls against real accounts. Escalating from earlier finding: this isn't just 'tenant_admin gets it when it should be 403' — the endpoint has no auth requirement whatsoever. Worth a decision on whether this is intended (a public health check) or a real gap.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): flag the 3 self-fixed-and-self-tested cases as pending independent re-test
Agreed process going forward: a fix and its verification shouldn't be done
by the same person alone. TC-020/060 (session revocation), TC-024/061
(health endpoint leak), and TC-025 (session cap) were all written and
live-tested by Claude with no second reviewer — flagged in each row's
Remarks so the tracker doesn't overstate confidence until the user has
independently re-tested them.

Scope reminder for this tracker going forward: only tenant_admin-scoped
features are tested here. super_admin-only features are covered
separately by another tester.
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -2192,7 +2192,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>Fixed in this session and verified live in one iteration — no further round needed. See TC-060 for the original bug-finding evidence.</t>
+          <t>PENDING INDEPENDENT RE-TEST: Claude wrote this fix and ran this test — same person, not independent verification. Agreed process going forward: the user (jithinjoseph-workspace) re-tests this separately before it's considered fully closed. | Fixed in this session and verified live in one iteration — no further round needed. See TC-060 for the original bug-finding evidence.</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>Fixed and re-verified. The test's original Expected Result ('Tenant Admin: 403 Forbidden') doesn't match what this architecture actually needs — recommend revising that expectation to 'unauthenticated: status only, authenticated: full data' rather than a 403.</t>
+          <t>PENDING INDEPENDENT RE-TEST: Claude wrote this fix and ran this test — same person, not independent verification. Agreed process going forward: the user (jithinjoseph-workspace) re-tests this separately before it's considered fully closed. | Fixed and re-verified. The test's original Expected Result ('Tenant Admin: 403 Forbidden') doesn't match what this architecture actually needs — recommend revising that expectation to 'unauthenticated: status only, authenticated: full data' rather than a 403.</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>Fixed and verified live: exact set of oldest sessions evicted, kept sessions unaffected, no stability impact.</t>
+          <t>PENDING INDEPENDENT RE-TEST: Claude wrote this fix and ran this test — same person, not independent verification. Agreed process going forward: the user (jithinjoseph-workspace) re-tests this separately before it's considered fully closed. | Fixed and verified live: exact set of oldest sessions evicted, kept sessions unaffected, no stability impact.</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="O61" s="4" t="inlineStr">
         <is>
-          <t>Deep re-test of TC-020 using a disposable throwaway account (qa-deep-test-01) instead of single one-shot calls against real accounts. Real, reproducible security bug: session revocation only clears one of the two session-key namespaces (ndr:session: vs provigil:session:) and is fully bypassable via /api/auth/refresh. Not something I changed — flagging for a fix decision. | FIXED and re-verified 2026-09-22, see TC-020.</t>
+          <t>PENDING INDEPENDENT RE-TEST: Claude wrote this fix and ran this test — same person, not independent verification. Agreed process going forward: the user (jithinjoseph-workspace) re-tests this separately before it's considered fully closed. | Deep re-test of TC-020 using a disposable throwaway account (qa-deep-test-01) instead of single one-shot calls against real accounts. Real, reproducible security bug: session revocation only clears one of the two session-key namespaces (ndr:session: vs provigil:session:) and is fully bypassable via /api/auth/refresh. Not something I changed — flagging for a fix decision. | FIXED and re-verified 2026-09-22, see TC-020.</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="O62" s="4" t="inlineStr">
         <is>
-          <t>Fixed and re-verified. The test's original Expected Result ('Tenant Admin: 403 Forbidden') doesn't match what this architecture actually needs — recommend revising that expectation to 'unauthenticated: status only, authenticated: full data' rather than a 403.</t>
+          <t>PENDING INDEPENDENT RE-TEST: Claude wrote this fix and ran this test — same person, not independent verification. Agreed process going forward: the user (jithinjoseph-workspace) re-tests this separately before it's considered fully closed. | Fixed and re-verified. The test's original Expected Result ('Tenant Admin: 403 Forbidden') doesn't match what this architecture actually needs — recommend revising that expectation to 'unauthenticated: status only, authenticated: full data' rather than a 403.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): re-verify TC-065 and TC-070 after the fix, including the self-caught gap
Both re-tested live after the rebuild(s):

- TC-065: assign+remove a real sensor on a disposable user, zero wait
  between remove and re-check (stricter than the original 3s-gap
  finding) - gone immediately.

- TC-070: tested in two rounds since the first rebuild only fixed the
  permission gate, not revoke_sensor_key()'s own mutation - caught that
  gap before reporting this done, fixed it, rebuilt again. Round 2:
  own-tenant revoke is immediately consistent (0s wait); a synthetic
  cross-tenant key (inserted directly via ClickHouse, since tenant_admin
  correctly can't create one for another tenant through the API) is
  correctly still rejected and confirmed unchanged afterward.

Both flagged pending independent re-test. 75 total: 70 Passed, 1
Blocked, 4 Failed (unchanged - same unbuilt super_admin features).
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -5671,7 +5671,7 @@
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
-          <t>Assign -&gt; HTTP 200, correctly appeared in the list. Remove -&gt; HTTP 200 {"removed":true}, but the assignment was STILL in the list on an immediate re-check. Traced to remove_sensor_assignment (clickhouse.rs:1719): 'ALTER TABLE ndr.user_sensor_assignments DELETE ...', the same async-mutation pattern as TC-062. Re-checked 3s later -&gt; correctly gone. Same finding cross-referenced, not a new distinct bug.</t>
+          <t>RE-TESTED after the fix (remove_sensor_assignment now uses SETTINGS mutations_sync=1, matching the pattern already used for ndr.users). Disposable analyst user, assigned a real sensor ('local-central'), then removed it, then read the assignments list with ZERO wait (no sleep at all between remove and re-check, unlike the original finding which used a 3s gap). Result: removal was HTTP 200, and the immediate re-check already showed it gone. Fixed.</t>
         </is>
       </c>
       <c r="K66" s="4" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="M66" s="4" t="inlineStr">
         <is>
-          <t>Claude (live API test, tenant-admin account, disposable data, https://localhost)</t>
+          <t>Claude (live API + direct ClickHouse check, post-fix rebuild, disposable/synthetic data)</t>
         </is>
       </c>
       <c r="N66" s="4" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="O66" s="4" t="inlineStr">
         <is>
-          <t>PENDING INDEPENDENT RE-TEST: Claude wrote/ran this alone — user re-test appreciated before fully closed. See TC-062 for the underlying pattern (async ClickHouse ALTER mutations).</t>
+          <t>PENDING INDEPENDENT RE-TEST: Claude wrote/ran this alone - user re-test appreciated. Fixed and re-verified with a 0-wait check (stricter than the original finding).</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
-          <t>HTTP 200 body {"message":"Forbidden: Only super_admin can revoke sensor keys"}. Confirmed in code (mod.rs, revoke_sensor_key_api): role check is strictly super_admin, no exception for the creator. Cleaned up the disposable key directly via ClickHouse since there is no tenant_admin-accessible path to do it.</t>
+          <t>RE-TESTED after the fix, in two rounds (the first rebuild only fixed the permission check, not the underlying mutation - caught and fixed in a second iteration before reporting this as done). Round 1: tenant_admin created their own sensor key, DELETE /api/sensor-keys/:id -&gt; HTTP 200 'Sensor key revoked', but an immediate list re-check still showed active=true (direct ClickHouse check confirmed the DB row itself was already active=0 - it was purely the same async-mutation read lag as TC-062/065, on revoke_sensor_key() specifically, which had been missed). Fixed by adding SETTINGS mutations_sync=1 to that query too. Round 2 (after rebuild): create-own-key -&gt; revoke -&gt; IMMEDIATE re-check (0s wait) -&gt; active:False, confirmed fixed. NEGATIVE path also tested: inserted a synthetic active sensor key owned by a different real tenant ('poi') directly via ClickHouse (since tenant_admin correctly cannot create one for another tenant), then tenant_admin attempted to revoke it -&gt; HTTP 200 body {"message":"Forbidden: cannot revoke another tenant's sensor key"}, and the row was confirmed still active=1 afterward (no effect). Synthetic test row cleaned up.</t>
         </is>
       </c>
       <c r="K71" s="4" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="M71" s="4" t="inlineStr">
         <is>
-          <t>Claude (live API test, tenant-admin account, disposable data, https://localhost)</t>
+          <t>Claude (live API + direct ClickHouse check, post-fix rebuild, disposable/synthetic data)</t>
         </is>
       </c>
       <c r="N71" s="4" t="inlineStr">
@@ -6088,7 +6088,7 @@
       </c>
       <c r="O71" s="4" t="inlineStr">
         <is>
-          <t>PENDING INDEPENDENT RE-TEST: Claude wrote/ran this alone — user re-test appreciated before fully closed. Not a bug - usability gap. A tenant_admin who creates a sensor key has no self-service way to revoke/rotate it; must ask a super_admin. Worth a product decision, not a security issue (asymmetric, not permissive).</t>
+          <t>PENDING INDEPENDENT RE-TEST: Claude wrote/ran this alone - user re-test appreciated. Fixed and re-verified: own-tenant revoke works immediately, cross-tenant revoke correctly still forbidden. First fix attempt was incomplete (permission check fixed, underlying mutation missed) - caught before reporting done, not after.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): TC-084 re-verified after rebuild - unauthenticated password reset now blocked
Re-ran the exact same attack that found this (POST /api/auth/reset-password,
no Authorization header, no old_password) against a fresh disposable
account on the rebuilt auth-service: now correctly returns
{"status":"error","message":"Unauthorized"}, and the original password
survived. Also confirmed the legitimate path (tenant_admin with a valid
session) still works, and a cross-tenant attempt safely returns
"User not found" rather than leaking or acting across tenants.

84 total: 79 Passed, 1 Blocked, 4 Failed (unchanged - unbuilt
super_admin features). No Critical or High severity findings remain
open.
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -7162,12 +7162,12 @@
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>Live, verified, zero-auth account takeover. Created qa-unauth-pwtest with password 'OriginalPw!2026a', confirmed it logs in. Called POST /api/auth/reset-password with NO Authorization header: {"username":"qa-unauth-pwtest","tenant_id":"default","new_password":"HackedByAnon!2026z"} -&gt; HTTP 200 {"message":"Password updated successfully"}. Confirmed original password now fails (401 Invalid credentials). Confirmed the attacker-set password now logs in successfully (full session issued, HTTP 200). This requires ZERO prior access - not a stolen token, not a low-privilege account, nothing - only knowing or guessing a username and tenant_id (tenant_id is very often 'default' or guessable/enumerable via other means).</t>
+          <t>RE-TESTED after the fix and rebuild, with the exact same attack as the original finding, on a fresh disposable account. Unauthenticated call (no Authorization header, no old_password) -&gt; HTTP 200 body {"status":"error","message":"Unauthorized"} - correctly rejected. Confirmed the original password still worked afterward (the attack had zero effect this time). Then verified the legitimate path still works: tenant_admin WITH a valid session token -&gt; 'Password updated successfully', new password logs in. Boundary check: tenant_admin attempting the reset with a DIFFERENT tenant_id ('poi') -&gt; 'User not found' (safe failure - the lookup is scoped to that tenant_id, so it can't be used to probe or act on another tenant's users).</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="L85" s="4" t="inlineStr">
@@ -7177,7 +7177,7 @@
       </c>
       <c r="M85" s="4" t="inlineStr">
         <is>
-          <t>Claude (live API test, disposable account, https://localhost)</t>
+          <t>Claude (live API test, disposable account, post-fix rebuild, https://localhost)</t>
         </is>
       </c>
       <c r="N85" s="4" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="O85" s="4" t="inlineStr">
         <is>
-          <t>CRITICAL, UNFIXED - reported, not yet fixed, pending explicit go-ahead before touching an authentication endpoint. This is more severe than anything else found this session (worse than the earlier session-revocation bug, which at least required holding a valid prior session). Anyone who can reach this API and knows/guesses a username+tenant_id can take over any account, including tenant_admin or super_admin, with no credentials whatsoever. The self-service path (old_password provided) IS correctly checked via bcrypt::verify - only the no-old_password 'admin reset' path is unauthenticated. The obviously correct fix is to add HeaderMap, extract claims, and require super_admin/tenant_admin (with tenant_admin restricted to their own tenant, matching every other admin-reset pattern already fixed this session), matching what the function's own comment already claims it does.</t>
+          <t>FIXED and re-verified 2026-09-22 with the identical attack that found it, plus the legitimate path and a cross-tenant boundary check. PENDING INDEPENDENT RE-TEST: user re-test appreciated given this was Critical severity.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): TC-089 re-verified after rebuild - empty domain and oversized note now rejected
Re-ran the exact inputs that originally found the gap (empty domain,
10,000-char note) against the rebuilt ndr-engine. Both now correctly
rejected at the API level; confirmed via follow-up list call that
neither was stored. Disposable test row cleaned up afterward.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -7558,12 +7558,12 @@
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>Both succeeded (HTTP 200) and were genuinely stored - confirmed the empty-domain row and the 10,000-char note both appeared in a follow-up list call. add_trusted_domain (mod.rs) has no is_empty()/length check on either field before the INSERT.</t>
+          <t>FIXED &amp; RE-VERIFIED post-rebuild (2026-09-22, ndr-engine containers recreated 11:10:14): re-ran the identical inputs that found the bug. Empty domain -&gt; {"error":"Domain is required"} HTTP 200 (app-level error). 10,000-char note -&gt; {"error":"Note is too long (max 500 characters)"} HTTP 200. Normal valid domain still succeeds. Follow-up GET /api/trusted-domains confirmed neither the empty-domain nor the oversized-note attempt was stored - only the disposable valid test row appeared, which was then removed via POST /api/trusted-domains/delete. No junk data left behind.</t>
         </is>
       </c>
       <c r="K90" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="L90" s="4" t="inlineStr">
@@ -7573,7 +7573,7 @@
       </c>
       <c r="M90" s="4" t="inlineStr">
         <is>
-          <t>Claude (live API test, disposable/synthetic data, https://localhost)</t>
+          <t>Claude (live API re-test, post-fix rebuild, https://localhost)</t>
         </is>
       </c>
       <c r="N90" s="4" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="O90" s="4" t="inlineStr">
         <is>
-          <t>PENDING INDEPENDENT RE-TEST: Claude wrote/ran this alone - user re-test appreciated. Real gap, not fixed (not asked to fix this one) - minor, doesn't grant unauthorized access, just lets junk/oversized data into the allowlist. Both test entries were cleaned up after confirming.</t>
+          <t>PENDING INDEPENDENT RE-TEST: fix in add_trusted_domain (mod.rs) - added is_empty()/253-char domain check and 500-char note cap. Re-tested with the exact inputs that originally found the gap; both now correctly rejected, storage confirmed clean via follow-up list. Same fixer/tester overlap as other entries - user re-test appreciated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): TC-081 fully verified - Save Settings clicked live, no side effects
Previously view-only (Apply Changes never clicked, since it writes real
tenant detection thresholds). Checked update_settings does a per-key
partial merge (not an overwrite) before clicking, then clicked with
identical values via real UI so the net effect is a no-op. Confirmed
UI success message and byte-identical GET /api/settings before/after,
including the adjacent ai_*/smtp_*/trusted_cloud_* fields the form
never touches.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -6905,7 +6905,7 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Logged in as tenant_admin</t>
+          <t>3. Click Apply Changes / Save Settings with unchanged values (verified backend does a per-key partial merge, not an overwrite, before clicking - update_settings only writes store/alert/critical/soar_threshold + sensitive_countries, never touches ai_*/smtp_*/trusted_cloud_* fields)</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
@@ -6921,12 +6921,12 @@
       </c>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>Real threshold values render, form is interactive</t>
+          <t>Real threshold values render, form is interactive Save Settings should persist correctly with no side effects on unrelated config.</t>
         </is>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>Rendered real values: Store=10, Alert=75, Critical=90, SOAR=75, plus a real 28-country sensitive-countries list with actual ISO codes. Sliders and an Apply Changes button present. 0 console errors. Did not click Apply Changes (would change real detection behavior for this tenant).</t>
+          <t>Rendered real values: Store=10, Alert=75, Critical=90, SOAR=75, plus a real 28-country sensitive-countries list with actual ISO codes. Sliders and an Apply Changes button present. 0 console errors. Did not click Apply Changes (would change real detection behavior for this tenant). UPDATED: clicked Save Settings via real UI (Playwright) with unchanged values. UI showed 'Settings saved' confirmation. GET /api/settings before/after are byte-identical - all 4 thresholds, sensitive_countries, AND the untouched ai_*/global_smtp_*/trusted_cloud_* fields all unchanged. 0 console errors. Full click-through workflow now verified, not just view.</t>
         </is>
       </c>
       <c r="K82" s="4" t="inlineStr">
@@ -6941,7 +6941,7 @@
       </c>
       <c r="M82" s="4" t="inlineStr">
         <is>
-          <t>Claude (real browser, headless Chromium via Playwright, https://localhost, tenant-admin account)</t>
+          <t>Claude (live UI test via Playwright, https://localhost)</t>
         </is>
       </c>
       <c r="N82" s="4" t="inlineStr">
@@ -6951,7 +6951,7 @@
       </c>
       <c r="O82" s="4" t="inlineStr">
         <is>
-          <t>PENDING INDEPENDENT RE-TEST: Claude drove this alone via browser automation - user click-through appreciated. Read-only check; did not submit a real threshold change.</t>
+          <t>PENDING INDEPENDENT RE-TEST: originally view-only (didn't click Apply, since it changes real tenant detection thresholds). Re-tested by checking update_settings does a safe partial merge first, then clicking with identical values so the net real-world effect is a no-op. Confirms the button works without risking a real threshold change.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): TC-080 fully verified - Start/Stop Monitoring exercised and reversed live
Previously view-only (didn't click Start/Stop, since it controls real
Zeek/Suricata/Arkime processes on the live sensor). Read the agent
handler (scripts/ndr-agent.py) first to confirm Vector/Telemetry is
never touched by this toggle, so a start-then-stop cycle is exactly
reversible. User approved the live toggle; clicked Start Monitoring
via real UI (confirmed all engines + Vector via API and UI), then
Stop Monitoring (confirmed restored to the exact original baseline
via API and UI). No lasting change to sensor state.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -6826,7 +6826,11 @@
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Logged in as tenant_admin</t>
+          <t>1. Navigate to Sensor Setup via sidebar
+2. Checked backend (/agent/start, /agent/stop in scripts/ndr-agent.py) first - confirmed they only control Zeek/Suricata/Arkime, never touch the separate Vector container, so start-&gt;stop is exactly reversible
+3. GET /api/agent-status for baseline
+4. Click Start Monitoring via real UI, confirm all 3 engines + Vector via API and UI
+5. Click Stop Monitoring via real UI, confirm restored to baseline via API and UI</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
@@ -6843,12 +6847,12 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>Real sensor status renders correctly</t>
+          <t>Real sensor status renders correctly; Start/Stop actually control the real engines and fully reverse</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>Rendered real data: Capture Interface 'eno1', '1/4 engines running', Agent-Z IDS STOPPED, Agent-S EVE STOPPED, Telemetry Pipeline RUNNING, PCAP Engine STOPPED - matches the actual state of this sensor. 0 console errors.</t>
+          <t>Rendered real data: Capture Interface 'eno1', '1/4 engines running', Agent-Z IDS STOPPED, Agent-S EVE STOPPED, Telemetry Pipeline RUNNING, PCAP Engine STOPPED - matches the actual state of this sensor. 0 console errors. UPDATED - full click-through now done. Baseline: agent-z stopped, agent-s stopped, arkime inactive, vector running (1/4). Clicked Start Monitoring -&gt; agent-status API and UI both confirmed agent-z/agent-s running, arkime active, vector still running (4/4, 'Monitoring Active'). Clicked Stop Monitoring -&gt; API and UI both confirmed restored to the exact original baseline (agent-z stopped, agent-s stopped, arkime inactive, vector still running throughout, 1/4). 0 console errors either direction.</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
@@ -6863,7 +6867,7 @@
       </c>
       <c r="M81" s="4" t="inlineStr">
         <is>
-          <t>Claude (real browser, headless Chromium via Playwright, https://localhost, tenant-admin account)</t>
+          <t>Claude (live UI test via Playwright + API verification, https://localhost)</t>
         </is>
       </c>
       <c r="N81" s="4" t="inlineStr">
@@ -6873,7 +6877,7 @@
       </c>
       <c r="O81" s="4" t="inlineStr">
         <is>
-          <t>PENDING INDEPENDENT RE-TEST: Claude drove this alone via browser automation - user click-through appreciated. Read-only check only. Start/Stop Monitoring buttons were NOT tested - would affect the real running sensor, same reasoning as TC-072/075.</t>
+          <t>PENDING INDEPENDENT RE-TEST: previously view-only (didn't click Start/Stop since it controls real IDS/EVE/PCAP processes on the live sensor, not app data). User explicitly approved a start-then-stop cycle. Read the agent's Python handler first to confirm Vector/Telemetry is never touched by this toggle before clicking, so the restore would be exact - confirmed via API before/after, not just visually. No lasting change to sensor state.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): TC-091 re-verified live after ndr-ui rebuild - dead link confirmed gone
Sidebar checked on both /tenant-admin/users and /tenant-admin/settings
post-rebuild - "PDF"/"Tenant Audit Report" no longer present, layout
clean with no gap left behind.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/NDR_Test_Case_Tracker.xlsx
+++ b/qa/NDR_Test_Case_Tracker.xlsx
@@ -7718,12 +7718,12 @@
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
-          <t>tenant-admin-layout.html has the markup ('PDF' badge + 'Tenant Audit Report' text) but tenant-admin-layout.ts has no matching click handler, method, or route reference at all - it is decorative only, does nothing when clicked.</t>
+          <t>tenant-admin-layout.html has the markup ('PDF' badge + 'Tenant Audit Report' text) but tenant-admin-layout.ts has no matching click handler, method, or route reference at all - it is decorative only, does nothing when clicked. RE-VERIFIED after ndr-ui rebuild (2026-09-22, container recreated 11:51:09): logged in live, checked sidebar on /tenant-admin/users and /tenant-admin/settings via DOM text extraction - 'PDF'/'Tenant Audit Report' no longer present anywhere in the sidebar. Screenshot confirms clean layout, nav ends cleanly after Support Center, no gap or leftover border artifact. 0 relevant console errors (one unrelated 429 from my own repeated test requests, not an app bug).</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="L92" s="4" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="M92" s="4" t="inlineStr">
         <is>
-          <t>Claude (source code review, no live test needed)</t>
+          <t>Claude (live UI re-test via Playwright, post-rebuild, https://localhost)</t>
         </is>
       </c>
       <c r="N92" s="4" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="O92" s="4" t="inlineStr">
         <is>
-          <t>PENDING INDEPENDENT RE-TEST: Claude wrote/ran this alone - user re-test appreciated. Not a bug exactly - a real feature that was apparently never wired up, or intentionally left as a visual placeholder. Not fixed (not asked to); flagging since it may confuse a real tenant admin expecting a working report download. Product decision (2026-09-22): remove the placeholder rather than build the report. Fix applied in tenant-admin-layout.html/.css (commit 11c668a), removes the dead &lt;span&gt; and orphaned CSS. NOT yet re-verified live - ndr-ui needs a rebuild first, then a UI check that the sidebar footer is gone and no layout gap is left behind.</t>
+          <t>PENDING INDEPENDENT RE-TEST: fix committed (11c668a), rebuilt by user, re-verified live - dead link confirmed gone, layout clean.</t>
         </is>
       </c>
     </row>

</xml_diff>